<commit_message>
Moderniza o tema escuro (paleta grafite, zebra, cabecalho e freeze)
- Nova paleta moderna (#18191D grafite azulado, acento #3B82F6),
  fonte Segoe UI, aplicada ao .thmx, ao suplemento VBA e a demo.
- Suplemento VBA: zebra via formatacao condicional (rapida em tabelas
  grandes), cabecalho com borda de acento, congelamento da 1a linha e
  grade sutil em vez de grade desligada.
- Demo e README atualizados com o novo visual.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Rah8Dke891DPSsn7hpcFi
</commit_message>
<xml_diff>
--- a/dist/DemoTemaEscuro.xlsx
+++ b/dist/DemoTemaEscuro.xlsx
@@ -26,14 +26,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="004FC3F7"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <color rgb="00F2F2F2"/>
+      <name val="Segoe UI"/>
+      <color rgb="00E4E6EB"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -45,21 +46,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002A2A2A"/>
+        <fgColor rgb="00212530"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E1E1E"/>
+        <fgColor rgb="001F2127"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002D2D30"/>
+        <fgColor rgb="0018191D"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -68,17 +69,22 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="medium">
+        <color rgb="003B82F6"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="003F3F3F"/>
+        <color rgb="002A2E38"/>
       </left>
       <right style="thin">
-        <color rgb="003F3F3F"/>
+        <color rgb="002A2E38"/>
       </right>
       <top style="thin">
-        <color rgb="003F3F3F"/>
+        <color rgb="002A2E38"/>
       </top>
       <bottom style="thin">
-        <color rgb="003F3F3F"/>
+        <color rgb="002A2E38"/>
       </bottom>
     </border>
   </borders>
@@ -90,11 +96,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -459,7 +465,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="004FC3F7"/>
+    <tabColor rgb="003B82F6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -472,7 +478,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Produto</t>
@@ -603,19 +609,43 @@
       <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Headset</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>349.9</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>18</v>
+      </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Cadeira</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Moveis</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1290</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>

</xml_diff>